<commit_message>
video02: críticas del guion (ronda 1), brief del showrunner; motor con zócalo (rotulo) y sin marca superpuesta; plantilla con matrices dinámicas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KsaNFb21PDHpGLAu3JPFa
</commit_message>
<xml_diff>
--- a/produccion/video02/plantilla/Distribuidora Sur.xlsx
+++ b/produccion/video02/plantilla/Distribuidora Sur.xlsx
@@ -15,6 +15,28 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1433,8 +1455,8 @@
       <c r="B2" s="3" t="n">
         <v>46296</v>
       </c>
-      <c r="D2">
-        <f>IFERROR(_xlfn._xlws.SORT(_xlfn._xlws.FILTER(_xlfn.CHOOSECOLS(Pedidos!A2:M13,3,11,10),Pedidos!M2:M13="Vencido"),3,-1),"Sin vencidos")</f>
+      <c r="D2" cm="1">
+        <f t="array" ref="D2">IFERROR(_xlfn._xlws.SORT(_xlfn._xlws.FILTER(_xlfn.CHOOSECOLS(Pedidos!A2:M13,3,11,10),Pedidos!M2:M13="Vencido"),3,-1),"Sin vencidos")</f>
         <v/>
       </c>
       <c r="E2" s="3" t="n"/>
@@ -1488,8 +1510,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>_xlfn._xlws.SORT(_xlfn.UNIQUE(Pedidos!C2:C13))</f>
+      <c r="A8" cm="1">
+        <f t="array" ref="A8">_xlfn._xlws.SORT(_xlfn.UNIQUE(Pedidos!C2:C13))</f>
         <v/>
       </c>
       <c r="B8">

</xml_diff>